<commit_message>
updating one copy and paste error
</commit_message>
<xml_diff>
--- a/data-raw/gtsummary_translated.xlsx
+++ b/data-raw/gtsummary_translated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sjobergd/Documents/GitHub/gtsummary/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7BC3EB0-4D26-CA43-B0CD-29E421BECF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3B4C68-BEF1-8642-A807-50379B447F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10180" yWindow="22360" windowWidth="30240" windowHeight="18880" xr2:uid="{24D5C74B-D2E9-42BC-9756-BFD64AB81539}"/>
   </bookViews>
@@ -3300,9 +3300,6 @@
     <t>Contrastes marginaux à la moyenne</t>
   </si>
   <si>
-    <t xml:space="preserve"> Contrastes marginaux aux moyennes marginales</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Contrastes marginaux</t>
   </si>
   <si>
@@ -3325,6 +3322,9 @@
   </si>
   <si>
     <t>test du khi-deux avec la correction du second ordre de Rao &amp; Scott</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Prédictions marginales aux moyennes marginales</t>
   </si>
 </sst>
 </file>
@@ -6069,7 +6069,7 @@
       <c r="E65"/>
       <c r="G65"/>
       <c r="L65" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="R65" t="s">
         <v>980</v>
@@ -6086,7 +6086,7 @@
       <c r="E66"/>
       <c r="G66"/>
       <c r="L66" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="R66" t="s">
         <v>981</v>
@@ -6103,7 +6103,7 @@
       <c r="E67"/>
       <c r="G67"/>
       <c r="L67" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="R67" t="s">
         <v>982</v>
@@ -6120,7 +6120,7 @@
       <c r="E68"/>
       <c r="G68"/>
       <c r="L68" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="R68" t="s">
         <v>983</v>
@@ -6137,7 +6137,7 @@
       <c r="E69"/>
       <c r="G69"/>
       <c r="L69" t="s">
-        <v>1053</v>
+        <v>1061</v>
       </c>
       <c r="R69" t="s">
         <v>984</v>
@@ -6154,7 +6154,7 @@
       <c r="E70"/>
       <c r="G70"/>
       <c r="L70" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="R70" t="s">
         <v>985</v>
@@ -7204,7 +7204,7 @@
       <c r="I92" s="9"/>
       <c r="J92" s="9"/>
       <c r="L92" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="Q92" t="s">
         <v>883</v>
@@ -7641,7 +7641,7 @@
         <v>274</v>
       </c>
       <c r="L102" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="O102" s="11" t="s">
         <v>704</v>
@@ -7677,7 +7677,7 @@
         <v>275</v>
       </c>
       <c r="L103" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="Q103" t="s">
         <v>873</v>

</xml_diff>